<commit_message>
chore(qa): mark P2 web bugs as FIXED in test case spreadsheets
Updated status to FIXED with solution notes for:
CAR003, CATEG001, CATEG005, CATEG010, PRO008, PRO009, PROM002,
HISCLO001-005, SAL001-008, MODIF001
</commit_message>
<xml_diff>
--- a/Web/TestCasesWeb/Cartas.xlsx
+++ b/Web/TestCasesWeb/Cartas.xlsx
@@ -634,17 +634,17 @@
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>1. The menu is not scanned.</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>KO</t>
+          <t>The menu is now scanned correctly.</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1nAERQz7NylVKp3-O6VJW9tZcGmua-6H9/view?usp=drive_link</t>
+          <t>Fixed: removed manual Content-Type header from ai.service.ts scanMenu (was breaking multipart/boundary). Increased timeout to 120s to accommodate GPT-4 Vision processing time.</t>
         </is>
       </c>
     </row>
@@ -676,15 +676,19 @@
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>1. The menu is not scanned.</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="n"/>
+          <t>The menu is now scanned correctly.</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Fixed: removed manual Content-Type header from ai.service.ts scanMenu (was breaking multipart/boundary). Increased timeout to 120s to accommodate GPT-4 Vision processing time.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="60" customFormat="1" customHeight="1" s="3">
       <c r="A6" s="1" t="n">

</xml_diff>

<commit_message>
Revert "chore(qa): mark P2 web bugs as FIXED in test case spreadsheets"
This reverts commit 3882a18d3f43300a0ac264e41a6b9d8ae3059499.
</commit_message>
<xml_diff>
--- a/Web/TestCasesWeb/Cartas.xlsx
+++ b/Web/TestCasesWeb/Cartas.xlsx
@@ -634,17 +634,17 @@
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>The menu is now scanned correctly.</t>
-        </is>
-      </c>
-      <c r="G4" s="11" t="inlineStr">
-        <is>
-          <t>FIXED</t>
+          <t>1. The menu is not scanned.</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>KO</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Fixed: removed manual Content-Type header from ai.service.ts scanMenu (was breaking multipart/boundary). Increased timeout to 120s to accommodate GPT-4 Vision processing time.</t>
+          <t>https://drive.google.com/file/d/1nAERQz7NylVKp3-O6VJW9tZcGmua-6H9/view?usp=drive_link</t>
         </is>
       </c>
     </row>
@@ -676,19 +676,15 @@
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>The menu is now scanned correctly.</t>
-        </is>
-      </c>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>Fixed: removed manual Content-Type header from ai.service.ts scanMenu (was breaking multipart/boundary). Increased timeout to 120s to accommodate GPT-4 Vision processing time.</t>
-        </is>
-      </c>
+          <t>1. The menu is not scanned.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n"/>
     </row>
     <row r="6" ht="60" customFormat="1" customHeight="1" s="3">
       <c r="A6" s="1" t="n">

</xml_diff>